<commit_message>
Added task an examples
</commit_message>
<xml_diff>
--- a/examples/data_nodes_intro.xlsx
+++ b/examples/data_nodes_intro.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zeeshan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jose/code/MainSequenceServerSide/excel-plugin/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{119B4FBE-F259-46BB-A271-F52BFF2B4A0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{942E2218-CA87-E54D-98F3-A66C4BFB51ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{37A25957-7996-1343-95F1-8493850F344D}"/>
+    <workbookView xWindow="4760" yWindow="11380" windowWidth="23240" windowHeight="13880" activeTab="1" xr2:uid="{37A25957-7996-1343-95F1-8493850F344D}"/>
   </bookViews>
   <sheets>
     <sheet name="simple_data_node" sheetId="1" r:id="rId1"/>
-    <sheet name="curve_expansion" sheetId="2" r:id="rId2"/>
+    <sheet name="Asset Detail" sheetId="3" r:id="rId2"/>
+    <sheet name="curve_expansion" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -59,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
   <si>
     <t>node_identifier</t>
   </si>
@@ -89,6 +90,51 @@
   </si>
   <si>
     <t>discount_curves</t>
+  </si>
+  <si>
+    <t>Assets</t>
+  </si>
+  <si>
+    <t>91_ACBE_24L</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 90_CBPF_48</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 90_CDMXCB_19</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 90_CHIACB_07</t>
+  </si>
+  <si>
+    <t>91_ACBE_24-2L</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 91_APEX_23</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 91_APEX_23-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 90_EDOMEX_22X</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 90_GCDMXCB_17X</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 90_GCDMXCB_18V</t>
+  </si>
+  <si>
+    <t>FAIL_ASSET</t>
+  </si>
+  <si>
+    <t>current_pricing_detail</t>
+  </si>
+  <si>
+    <t>current_snapshot</t>
+  </si>
+  <si>
+    <t>name</t>
   </si>
 </sst>
 </file>
@@ -133,10 +179,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -485,6 +532,9 @@
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
   <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions val="1"/>
+    </a:ext>
     <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
       <we:customFunctionIdList>
         <we:customFunctionIds>_xldudf_MAINSEQUENCE_GET_DATA</we:customFunctionIds>
@@ -496,14 +546,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1226C041-A466-F740-911C-1A43C4B5C3DD}">
-  <dimension ref="B9:H19"/>
-  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15.6"/>
+  <dimension ref="B9:AK19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
-    <col min="2" max="2" width="16.44921875" customWidth="1"/>
-    <col min="3" max="3" width="22.09765625" customWidth="1"/>
+    <col min="2" max="2" width="16.5" customWidth="1"/>
+    <col min="3" max="3" width="22.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="9" spans="2:8">
+    <row r="9" spans="2:37">
       <c r="B9" t="s">
         <v>0</v>
       </c>
@@ -511,54 +561,891 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="2:8">
+    <row r="10" spans="2:37">
       <c r="B10" t="s">
         <v>1</v>
       </c>
       <c r="C10" s="1">
-        <f>DATE(2025,10,20)</f>
-        <v>45950</v>
-      </c>
-    </row>
-    <row r="11" spans="2:8">
+        <f>DATE(2022,6,20)</f>
+        <v>44732</v>
+      </c>
+    </row>
+    <row r="11" spans="2:37">
       <c r="B11" t="s">
         <v>2</v>
       </c>
       <c r="C11" s="1">
-        <f>DATE(2025,11,15)</f>
-        <v>45976</v>
+        <f>DATE(2022,6,25)</f>
+        <v>44737</v>
       </c>
       <c r="G11" t="str" cm="1">
-        <f t="array" ref="G11:H11">_xldudf_MAINSEQUENCE_GET_DATA(C10, C11, B18:B19,C9, TRUE, TRUE, 500, 0,"null")</f>
-        <v>Error</v>
+        <f t="array" ref="G11:AK19">_xldudf_MAINSEQUENCE_GET_DATA(C10, C11, B18:B19,C9, TRUE, TRUE, 500, 0,"null")</f>
+        <v>time_index</v>
       </c>
       <c r="H11" t="str">
-        <v>No refresh token available</v>
-      </c>
-    </row>
-    <row r="12" spans="2:8">
+        <v>unique_identifier</v>
+      </c>
+      <c r="I11" t="str">
+        <v>secid</v>
+      </c>
+      <c r="J11" t="str">
+        <v>tradedate</v>
+      </c>
+      <c r="K11" t="str">
+        <v>ticker</v>
+      </c>
+      <c r="L11" t="str">
+        <v>name</v>
+      </c>
+      <c r="M11" t="str">
+        <v>primaryexchange</v>
+      </c>
+      <c r="N11" t="str">
+        <v>isin</v>
+      </c>
+      <c r="O11" t="str">
+        <v>open</v>
+      </c>
+      <c r="P11" t="str">
+        <v>opensize</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>high</v>
+      </c>
+      <c r="R11" t="str">
+        <v>hightime</v>
+      </c>
+      <c r="S11" t="str">
+        <v>low</v>
+      </c>
+      <c r="T11" t="str">
+        <v>lowtime</v>
+      </c>
+      <c r="U11" t="str">
+        <v>close</v>
+      </c>
+      <c r="V11" t="str">
+        <v>closesize</v>
+      </c>
+      <c r="W11" t="str">
+        <v>listedmarkethoursvolume</v>
+      </c>
+      <c r="X11" t="str">
+        <v>listedmarkethourstrades</v>
+      </c>
+      <c r="Y11" t="str">
+        <v>volume</v>
+      </c>
+      <c r="Z11" t="str">
+        <v>listedtotaltrades</v>
+      </c>
+      <c r="AA11" t="str">
+        <v>finramarkethoursvolume</v>
+      </c>
+      <c r="AB11" t="str">
+        <v>finramarkethourstrades</v>
+      </c>
+      <c r="AC11" t="str">
+        <v>finratotalvolume</v>
+      </c>
+      <c r="AD11" t="str">
+        <v>finratotaltrades</v>
+      </c>
+      <c r="AE11" t="str">
+        <v>cumulativepricefactor</v>
+      </c>
+      <c r="AF11" t="str">
+        <v>cumulativevolumefactor</v>
+      </c>
+      <c r="AG11" t="str">
+        <v>adjustmentfactor</v>
+      </c>
+      <c r="AH11" t="str">
+        <v>adjustmentreason</v>
+      </c>
+      <c r="AI11" t="str">
+        <v>vwap</v>
+      </c>
+      <c r="AJ11" t="str">
+        <v>dailyvwap</v>
+      </c>
+      <c r="AK11" t="str">
+        <v>open_time</v>
+      </c>
+    </row>
+    <row r="12" spans="2:37">
       <c r="B12" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="13" spans="2:8">
+      <c r="G12" t="str">
+        <v>2022-06-21T20:04:21.062Z</v>
+      </c>
+      <c r="H12" t="str">
+        <v>BBG000BS7KS3</v>
+      </c>
+      <c r="I12" t="str">
+        <v>32840</v>
+      </c>
+      <c r="J12" t="str">
+        <v>20220621</v>
+      </c>
+      <c r="K12" t="str">
+        <v>TAP</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Molson Coors Beverage Company</v>
+      </c>
+      <c r="M12" t="str">
+        <v>NYSE</v>
+      </c>
+      <c r="N12" t="str">
+        <v>US60871R2094</v>
+      </c>
+      <c r="O12" t="str">
+        <v>49.89</v>
+      </c>
+      <c r="P12" t="str">
+        <v>33463</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>52.37</v>
+      </c>
+      <c r="R12" t="str">
+        <v>15:54:27.864126976</v>
+      </c>
+      <c r="S12" t="str">
+        <v>49.86</v>
+      </c>
+      <c r="T12" t="str">
+        <v>09:30:01.135874560</v>
+      </c>
+      <c r="U12" t="str">
+        <v>52.21</v>
+      </c>
+      <c r="V12" t="str">
+        <v>225645</v>
+      </c>
+      <c r="W12" t="str">
+        <v>1215254</v>
+      </c>
+      <c r="X12" t="str">
+        <v>19139</v>
+      </c>
+      <c r="Y12" t="str">
+        <v>1218571</v>
+      </c>
+      <c r="Z12" t="str">
+        <v>19178</v>
+      </c>
+      <c r="AA12" t="str">
+        <v>504367</v>
+      </c>
+      <c r="AB12" t="str">
+        <v>5549</v>
+      </c>
+      <c r="AC12" t="str">
+        <v>536759</v>
+      </c>
+      <c r="AD12" t="str">
+        <v>5588</v>
+      </c>
+      <c r="AE12" t="str">
+        <v>2.8146466416</v>
+      </c>
+      <c r="AF12" t="str">
+        <v>2</v>
+      </c>
+      <c r="AG12" t="str">
+        <v/>
+      </c>
+      <c r="AH12" t="str">
+        <v/>
+      </c>
+      <c r="AI12" t="str">
+        <v>51.57</v>
+      </c>
+      <c r="AJ12" t="str">
+        <v>51.58</v>
+      </c>
+      <c r="AK12" t="str">
+        <v>1655818201002417400</v>
+      </c>
+    </row>
+    <row r="13" spans="2:37">
       <c r="B13" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="17" spans="2:2">
+      <c r="G13" t="str">
+        <v>2022-06-21T20:04:23.799Z</v>
+      </c>
+      <c r="H13" t="str">
+        <v>BBG000BY29C7</v>
+      </c>
+      <c r="I13" t="str">
+        <v>35035</v>
+      </c>
+      <c r="J13" t="str">
+        <v>20220621</v>
+      </c>
+      <c r="K13" t="str">
+        <v>TPR</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Tapestry Inc</v>
+      </c>
+      <c r="M13" t="str">
+        <v>NYSE</v>
+      </c>
+      <c r="N13" t="str">
+        <v>US8760301072</v>
+      </c>
+      <c r="O13" t="str">
+        <v>32.86</v>
+      </c>
+      <c r="P13" t="str">
+        <v>34525</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>33.12</v>
+      </c>
+      <c r="R13" t="str">
+        <v>09:31:07.155833088</v>
+      </c>
+      <c r="S13" t="str">
+        <v>31.79</v>
+      </c>
+      <c r="T13" t="str">
+        <v>09:45:50.420385280</v>
+      </c>
+      <c r="U13" t="str">
+        <v>32.15</v>
+      </c>
+      <c r="V13" t="str">
+        <v>516277</v>
+      </c>
+      <c r="W13" t="str">
+        <v>2350872</v>
+      </c>
+      <c r="X13" t="str">
+        <v>26708</v>
+      </c>
+      <c r="Y13" t="str">
+        <v>2351529</v>
+      </c>
+      <c r="Z13" t="str">
+        <v>26722</v>
+      </c>
+      <c r="AA13" t="str">
+        <v>919073</v>
+      </c>
+      <c r="AB13" t="str">
+        <v>8374</v>
+      </c>
+      <c r="AC13" t="str">
+        <v>1234117</v>
+      </c>
+      <c r="AD13" t="str">
+        <v>8417</v>
+      </c>
+      <c r="AE13" t="str">
+        <v>1.4005522671</v>
+      </c>
+      <c r="AF13" t="str">
+        <v>1</v>
+      </c>
+      <c r="AG13" t="str">
+        <v/>
+      </c>
+      <c r="AH13" t="str">
+        <v/>
+      </c>
+      <c r="AI13" t="str">
+        <v>32.21</v>
+      </c>
+      <c r="AJ13" t="str">
+        <v>32.21</v>
+      </c>
+      <c r="AK13" t="str">
+        <v>1655818200795210200</v>
+      </c>
+    </row>
+    <row r="14" spans="2:37">
+      <c r="G14" t="str">
+        <v>2022-06-22T20:04:22.187Z</v>
+      </c>
+      <c r="H14" t="str">
+        <v>BBG000BS7KS3</v>
+      </c>
+      <c r="I14" t="str">
+        <v>32840</v>
+      </c>
+      <c r="J14" t="str">
+        <v>20220622</v>
+      </c>
+      <c r="K14" t="str">
+        <v>TAP</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Molson Coors Beverage Company</v>
+      </c>
+      <c r="M14" t="str">
+        <v>NYSE</v>
+      </c>
+      <c r="N14" t="str">
+        <v>US60871R2094</v>
+      </c>
+      <c r="O14" t="str">
+        <v>51.59</v>
+      </c>
+      <c r="P14" t="str">
+        <v>16534</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>52.95</v>
+      </c>
+      <c r="R14" t="str">
+        <v>15:54:29.427121920</v>
+      </c>
+      <c r="S14" t="str">
+        <v>51.5</v>
+      </c>
+      <c r="T14" t="str">
+        <v>09:30:55.435228928</v>
+      </c>
+      <c r="U14" t="str">
+        <v>52.72</v>
+      </c>
+      <c r="V14" t="str">
+        <v>228798</v>
+      </c>
+      <c r="W14" t="str">
+        <v>893884</v>
+      </c>
+      <c r="X14" t="str">
+        <v>14950</v>
+      </c>
+      <c r="Y14" t="str">
+        <v>893884</v>
+      </c>
+      <c r="Z14" t="str">
+        <v>14950</v>
+      </c>
+      <c r="AA14" t="str">
+        <v>360055</v>
+      </c>
+      <c r="AB14" t="str">
+        <v>4710</v>
+      </c>
+      <c r="AC14" t="str">
+        <v>397756</v>
+      </c>
+      <c r="AD14" t="str">
+        <v>4756</v>
+      </c>
+      <c r="AE14" t="str">
+        <v>2.8146466416</v>
+      </c>
+      <c r="AF14" t="str">
+        <v>2</v>
+      </c>
+      <c r="AG14" t="str">
+        <v/>
+      </c>
+      <c r="AH14" t="str">
+        <v/>
+      </c>
+      <c r="AI14" t="str">
+        <v>52.57</v>
+      </c>
+      <c r="AJ14" t="str">
+        <v>52.58</v>
+      </c>
+      <c r="AK14" t="str">
+        <v>1655904601046734600</v>
+      </c>
+    </row>
+    <row r="15" spans="2:37">
+      <c r="G15" t="str">
+        <v>2022-06-22T20:04:26.643Z</v>
+      </c>
+      <c r="H15" t="str">
+        <v>BBG000BY29C7</v>
+      </c>
+      <c r="I15" t="str">
+        <v>35035</v>
+      </c>
+      <c r="J15" t="str">
+        <v>20220622</v>
+      </c>
+      <c r="K15" t="str">
+        <v>TPR</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Tapestry Inc</v>
+      </c>
+      <c r="M15" t="str">
+        <v>NYSE</v>
+      </c>
+      <c r="N15" t="str">
+        <v>US8760301072</v>
+      </c>
+      <c r="O15" t="str">
+        <v>31.61</v>
+      </c>
+      <c r="P15" t="str">
+        <v>33525</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>32.09</v>
+      </c>
+      <c r="R15" t="str">
+        <v>09:33:14.717302016</v>
+      </c>
+      <c r="S15" t="str">
+        <v>30.97</v>
+      </c>
+      <c r="T15" t="str">
+        <v>15:41:12.881224448</v>
+      </c>
+      <c r="U15" t="str">
+        <v>31.11</v>
+      </c>
+      <c r="V15" t="str">
+        <v>686094</v>
+      </c>
+      <c r="W15" t="str">
+        <v>3032012</v>
+      </c>
+      <c r="X15" t="str">
+        <v>32030</v>
+      </c>
+      <c r="Y15" t="str">
+        <v>3032247</v>
+      </c>
+      <c r="Z15" t="str">
+        <v>32037</v>
+      </c>
+      <c r="AA15" t="str">
+        <v>1010946</v>
+      </c>
+      <c r="AB15" t="str">
+        <v>8780</v>
+      </c>
+      <c r="AC15" t="str">
+        <v>1162394</v>
+      </c>
+      <c r="AD15" t="str">
+        <v>8826</v>
+      </c>
+      <c r="AE15" t="str">
+        <v>1.4005522671</v>
+      </c>
+      <c r="AF15" t="str">
+        <v>1</v>
+      </c>
+      <c r="AG15" t="str">
+        <v/>
+      </c>
+      <c r="AH15" t="str">
+        <v/>
+      </c>
+      <c r="AI15" t="str">
+        <v>31.34</v>
+      </c>
+      <c r="AJ15" t="str">
+        <v>31.33</v>
+      </c>
+      <c r="AK15" t="str">
+        <v>1655904600699598300</v>
+      </c>
+    </row>
+    <row r="16" spans="2:37">
+      <c r="G16" t="str">
+        <v>2022-06-23T20:04:00.471Z</v>
+      </c>
+      <c r="H16" t="str">
+        <v>BBG000BS7KS3</v>
+      </c>
+      <c r="I16" t="str">
+        <v>32840</v>
+      </c>
+      <c r="J16" t="str">
+        <v>20220623</v>
+      </c>
+      <c r="K16" t="str">
+        <v>TAP</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Molson Coors Beverage Company</v>
+      </c>
+      <c r="M16" t="str">
+        <v>NYSE</v>
+      </c>
+      <c r="N16" t="str">
+        <v>US60871R2094</v>
+      </c>
+      <c r="O16" t="str">
+        <v>52.72</v>
+      </c>
+      <c r="P16" t="str">
+        <v>14080</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>53.87</v>
+      </c>
+      <c r="R16" t="str">
+        <v>15:52:00.758303232</v>
+      </c>
+      <c r="S16" t="str">
+        <v>52.61</v>
+      </c>
+      <c r="T16" t="str">
+        <v>09:30:17.684049152</v>
+      </c>
+      <c r="U16" t="str">
+        <v>53.8</v>
+      </c>
+      <c r="V16" t="str">
+        <v>211103</v>
+      </c>
+      <c r="W16" t="str">
+        <v>927269</v>
+      </c>
+      <c r="X16" t="str">
+        <v>13302</v>
+      </c>
+      <c r="Y16" t="str">
+        <v>927703</v>
+      </c>
+      <c r="Z16" t="str">
+        <v>13314</v>
+      </c>
+      <c r="AA16" t="str">
+        <v>539338</v>
+      </c>
+      <c r="AB16" t="str">
+        <v>3613</v>
+      </c>
+      <c r="AC16" t="str">
+        <v>586131</v>
+      </c>
+      <c r="AD16" t="str">
+        <v>3645</v>
+      </c>
+      <c r="AE16" t="str">
+        <v>2.8146466416</v>
+      </c>
+      <c r="AF16" t="str">
+        <v>2</v>
+      </c>
+      <c r="AG16" t="str">
+        <v/>
+      </c>
+      <c r="AH16" t="str">
+        <v/>
+      </c>
+      <c r="AI16" t="str">
+        <v>53.43</v>
+      </c>
+      <c r="AJ16" t="str">
+        <v>53.44</v>
+      </c>
+      <c r="AK16" t="str">
+        <v>1655991000874342400</v>
+      </c>
+    </row>
+    <row r="17" spans="2:37">
       <c r="B17" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="18" spans="2:2">
+      <c r="G17" t="str">
+        <v>2022-06-23T20:04:01.776Z</v>
+      </c>
+      <c r="H17" t="str">
+        <v>BBG000BY29C7</v>
+      </c>
+      <c r="I17" t="str">
+        <v>35035</v>
+      </c>
+      <c r="J17" t="str">
+        <v>20220623</v>
+      </c>
+      <c r="K17" t="str">
+        <v>TPR</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Tapestry Inc</v>
+      </c>
+      <c r="M17" t="str">
+        <v>NYSE</v>
+      </c>
+      <c r="N17" t="str">
+        <v>US8760301072</v>
+      </c>
+      <c r="O17" t="str">
+        <v>31.4</v>
+      </c>
+      <c r="P17" t="str">
+        <v>28575</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>32.17</v>
+      </c>
+      <c r="R17" t="str">
+        <v>15:41:03.035004928</v>
+      </c>
+      <c r="S17" t="str">
+        <v>31.2</v>
+      </c>
+      <c r="T17" t="str">
+        <v>09:54:51.274644736</v>
+      </c>
+      <c r="U17" t="str">
+        <v>32.09</v>
+      </c>
+      <c r="V17" t="str">
+        <v>231128</v>
+      </c>
+      <c r="W17" t="str">
+        <v>2236421</v>
+      </c>
+      <c r="X17" t="str">
+        <v>25920</v>
+      </c>
+      <c r="Y17" t="str">
+        <v>2236426</v>
+      </c>
+      <c r="Z17" t="str">
+        <v>25922</v>
+      </c>
+      <c r="AA17" t="str">
+        <v>861624</v>
+      </c>
+      <c r="AB17" t="str">
+        <v>6313</v>
+      </c>
+      <c r="AC17" t="str">
+        <v>1272771</v>
+      </c>
+      <c r="AD17" t="str">
+        <v>6348</v>
+      </c>
+      <c r="AE17" t="str">
+        <v>1.4005522671</v>
+      </c>
+      <c r="AF17" t="str">
+        <v>1</v>
+      </c>
+      <c r="AG17" t="str">
+        <v/>
+      </c>
+      <c r="AH17" t="str">
+        <v/>
+      </c>
+      <c r="AI17" t="str">
+        <v>31.77</v>
+      </c>
+      <c r="AJ17" t="str">
+        <v>31.8</v>
+      </c>
+      <c r="AK17" t="str">
+        <v>1655991037299965000</v>
+      </c>
+    </row>
+    <row r="18" spans="2:37">
       <c r="B18" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="19" spans="2:2">
+      <c r="G18" t="str">
+        <v>2022-06-24T20:04:30.414Z</v>
+      </c>
+      <c r="H18" t="str">
+        <v>BBG000BY29C7</v>
+      </c>
+      <c r="I18" t="str">
+        <v>35035</v>
+      </c>
+      <c r="J18" t="str">
+        <v>20220624</v>
+      </c>
+      <c r="K18" t="str">
+        <v>TPR</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Tapestry Inc</v>
+      </c>
+      <c r="M18" t="str">
+        <v>NYSE</v>
+      </c>
+      <c r="N18" t="str">
+        <v>US8760301072</v>
+      </c>
+      <c r="O18" t="str">
+        <v>32.68</v>
+      </c>
+      <c r="P18" t="str">
+        <v>22426</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>33.62</v>
+      </c>
+      <c r="R18" t="str">
+        <v>11:39:43.900403200</v>
+      </c>
+      <c r="S18" t="str">
+        <v>32.56</v>
+      </c>
+      <c r="T18" t="str">
+        <v>09:31:01.988304384</v>
+      </c>
+      <c r="U18" t="str">
+        <v>33.33</v>
+      </c>
+      <c r="V18" t="str">
+        <v>935312</v>
+      </c>
+      <c r="W18" t="str">
+        <v>2766645</v>
+      </c>
+      <c r="X18" t="str">
+        <v>21183</v>
+      </c>
+      <c r="Y18" t="str">
+        <v>2766953</v>
+      </c>
+      <c r="Z18" t="str">
+        <v>21196</v>
+      </c>
+      <c r="AA18" t="str">
+        <v>926219</v>
+      </c>
+      <c r="AB18" t="str">
+        <v>7601</v>
+      </c>
+      <c r="AC18" t="str">
+        <v>1235246</v>
+      </c>
+      <c r="AD18" t="str">
+        <v>7645</v>
+      </c>
+      <c r="AE18" t="str">
+        <v>1.4005522671</v>
+      </c>
+      <c r="AF18" t="str">
+        <v>1</v>
+      </c>
+      <c r="AG18" t="str">
+        <v/>
+      </c>
+      <c r="AH18" t="str">
+        <v/>
+      </c>
+      <c r="AI18" t="str">
+        <v>33.32</v>
+      </c>
+      <c r="AJ18" t="str">
+        <v>33.32</v>
+      </c>
+      <c r="AK18" t="str">
+        <v>1656077400750235400</v>
+      </c>
+    </row>
+    <row r="19" spans="2:37">
       <c r="B19" t="s">
         <v>5</v>
+      </c>
+      <c r="G19" t="str">
+        <v>2022-06-24T20:04:32.635Z</v>
+      </c>
+      <c r="H19" t="str">
+        <v>BBG000BS7KS3</v>
+      </c>
+      <c r="I19" t="str">
+        <v>32840</v>
+      </c>
+      <c r="J19" t="str">
+        <v>20220624</v>
+      </c>
+      <c r="K19" t="str">
+        <v>TAP</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Molson Coors Beverage Company</v>
+      </c>
+      <c r="M19" t="str">
+        <v>NYSE</v>
+      </c>
+      <c r="N19" t="str">
+        <v>US60871R2094</v>
+      </c>
+      <c r="O19" t="str">
+        <v>54.22</v>
+      </c>
+      <c r="P19" t="str">
+        <v>13512</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>56.13</v>
+      </c>
+      <c r="R19" t="str">
+        <v>13:31:28.540152064</v>
+      </c>
+      <c r="S19" t="str">
+        <v>53.92</v>
+      </c>
+      <c r="T19" t="str">
+        <v>09:41:23.891128064</v>
+      </c>
+      <c r="U19" t="str">
+        <v>55.77</v>
+      </c>
+      <c r="V19" t="str">
+        <v>381339</v>
+      </c>
+      <c r="W19" t="str">
+        <v>1148886</v>
+      </c>
+      <c r="X19" t="str">
+        <v>15687</v>
+      </c>
+      <c r="Y19" t="str">
+        <v>1149258</v>
+      </c>
+      <c r="Z19" t="str">
+        <v>15698</v>
+      </c>
+      <c r="AA19" t="str">
+        <v>362077</v>
+      </c>
+      <c r="AB19" t="str">
+        <v>4628</v>
+      </c>
+      <c r="AC19" t="str">
+        <v>512730</v>
+      </c>
+      <c r="AD19" t="str">
+        <v>4656</v>
+      </c>
+      <c r="AE19" t="str">
+        <v>2.8146466416</v>
+      </c>
+      <c r="AF19" t="str">
+        <v>2</v>
+      </c>
+      <c r="AG19" t="str">
+        <v/>
+      </c>
+      <c r="AH19" t="str">
+        <v/>
+      </c>
+      <c r="AI19" t="str">
+        <v>55.54</v>
+      </c>
+      <c r="AJ19" t="str">
+        <v>55.56</v>
+      </c>
+      <c r="AK19" t="str">
+        <v>1656077400894880300</v>
       </c>
     </row>
   </sheetData>
@@ -567,13 +1454,113 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ED7E505-7C51-F949-84FB-580C9CDDFA81}">
+  <dimension ref="C8:I19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="3" max="3" width="18.5" customWidth="1"/>
+    <col min="8" max="8" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="8" spans="3:9">
+      <c r="C8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="3:9">
+      <c r="C9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="e" cm="1">
+        <f t="array" aca="1" ref="D9" ca="1">GET_ASSET(C9)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="F9" t="e" cm="1">
+        <f t="array" aca="1" ref="F9" ca="1">INDEX(PARSEJSON($D9), F8)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="H9" t="e" cm="1">
+        <f t="array" aca="1" ref="H9" ca="1">INDEX(PARSEJSON($D9), H8)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="I9" t="e" cm="1">
+        <f t="array" aca="1" ref="I9" ca="1">INDEX(PARSEJSON($H9), I8)</f>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="10" spans="3:9">
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="3:9">
+      <c r="C11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="3:9">
+      <c r="C12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="3:9">
+      <c r="C13" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="3:9">
+      <c r="C14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="3:9">
+      <c r="C15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="3:9">
+      <c r="C16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3">
+      <c r="C17" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="3:3">
+      <c r="C18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="3:3">
+      <c r="C19" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65FFC575-72C0-7144-B736-5CD1880658C9}">
   <dimension ref="B9:H20"/>
-  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15.6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="6" max="6" width="22.3984375" customWidth="1"/>
-    <col min="7" max="7" width="32.69921875" customWidth="1"/>
+    <col min="6" max="6" width="22.33203125" customWidth="1"/>
+    <col min="7" max="7" width="32.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="9" spans="2:8">

</xml_diff>